<commit_message>
feat(F-NAR-019): ATOM-AUT.RAN.001-07 La vache d'or
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.RAN.001-07.xlsx
+++ b/stories/arbres/ATOM-AUT.RAN.001-07.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Aniss veut l'histoire au lit avec sa vache en bois. Le mouton et les perles la recouvrent. Il cherche, met bêtes et perles dans la caisse. La vache apparaît. Maman raconte.</t>
+          <t>La fenêtre laisse entrer la terre mouillée. Un papillon frappe la vitre. Sur le flanc de la vache, un éclat de lampe brille. Aniss veut le collier et l'histoire au lit, maintenant. Le cheval bascule : le mouton recouvre la vache. Il cherche sous le lit, dans le cercle : rien. Il prend tout d'un coup : les bêtes s'éparpillent. Il refuse de foncer, pose le cheval, retrouve la vache. Sur l'oreiller, l'éclat de lampe tient au flanc.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un papillon de nuit frappe la vitre. Tout doucement. L'air sent la terre mouillée. La fenêtre est un peu ouverte. Le plancher craque. Le soir est calme. Oui, un petit soir doux. Des animaux en bois attendent en rang. La vache est lisse. Le cheval sent le bois. En ce moment, Aniss est à genoux. Il est dans le rond d'or de la lampe. C'est une ferme, maman. Une ferme sur le tapis. Aniss pose la vache. Il pose le cheval. Les bêtes tapent doucement. Il pose aussi un mouton. Elles sont bien, tes bêtes. La vache mange, papa. Et le mouton ? Il dort près de la vache. Aniss sort des perles. Elles sont rondes. Elles brillent un peu dans la lampe. Je fais un collier pour la vache. Un collier tout doux. Aniss enfile une perle. Puis une autre perle. Les perles font un tout petit bruit. Il pose le collier sur le cou de la vache. Elle est belle. Oui, elle est belle. Après, tu racontes une histoire, maman ? Oui, près de toi, au lit. La vache vient aussi. Maman s'approche du tapis. Le cheval bascule. Une perle roule. Le mouton glisse sur la vache. Oh. La ferme a bougé. Où est ma vache ? Sous le lit, peut-être ? Aniss se penche dans l'ombre. Le bois du lit est froid. Pas de vache. Dans le rond d'or ? Il cherche au milieu de la lumière. Des perles, le cheval, le mouton. Elle est perdue. J'ai besoin d'un petit coin, pour raconter. Je veux voir dessous. Aniss prend le cheval. Il le pose dans la caisse. Toc. La caisse sent le bois.</t>
+          <t>La fenêtre laisse entrer un air de terre mouillée, un peu froid. Un papillon de nuit se pose, puis frappe la vitre du bout des ailes. Sa silhouette tremble un peu, sur le tapis. Tu entends les ailes, Aniss ? Oui, maman. Le plancher craque sous le pas de papa. La lampe ronde est allumée. Elle chauffe le bois des bêtes, une à une. Sur le flanc de la vache, un éclat de lampe brille. Il est tout petit, papa. C'est un éclat de lampe. La vache est lisse, un peu chaude sous le doigt. Le cheval sent le bois, sec et clair. C'est une ferme, maman. Une ferme sur le tapis. En ce moment, Aniss pose la vache au milieu du tapis. Il pose le cheval à côté, tap. Le mouton vient après, laine peinte, un peu rêche. Elles sont bien, tes bêtes. La vache mange, papa. Et le mouton ? Il dort près de la vache. Aniss sort des perles d'une coupelle. Elles sont rondes, un peu froides dans la paume. Je fais un collier, maintenant ! Pour la vache d'or ? Oui, et après l'histoire au lit. Aniss enfile une perle, clic. Puis une autre, clic, contre la première. Les perles font un tout petit bruit. Il pose le collier sur le cou de la vache. Elle est belle. Oui, elle est belle. L'histoire, maintenant, maman ! Près de toi, au lit ? La vache vient aussi. Maman s'approche du tapis, trop près des bêtes. Le cheval bascule. Une perle roule sous le lit. Le mouton glisse sur la vache, et la cache. Oh. La ferme a bougé. Où est ma vache ? Sous le lit, peut-être ? Aniss se penche dans l'ombre, près du bois. Le bois du lit est froid, un peu rugueux. Pas de vache. Dans le cercle de la lampe ? Il cherche au milieu de la lumière ronde. Des perles, le cheval, le mouton. Elle est perdue. Je prends tout, d'un coup ! Il saisit le cheval et le mouton trop vite. Les perles glissent entre ses doigts. Le tapis disparaît sous les bêtes. Ça ne veut pas, papa. Ses épaules tombent un peu. Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tu regardes sous les bêtes ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un papillon de nuit frappe la vitre. Tout doucement. L'air sent la terre mouillée. La fenêtre est un peu ouverte. Le plancher craque. Le soir est calme. Oui, un petit soir doux. Des animaux en bois attendent en rang. La vache est lisse. Le cheval sent le bois. En ce moment, Aniss est à genoux. Il est dans le rond d'or de la lampe. C'est une ferme, maman. Une ferme sur le tapis. Aniss pose la vache. Il pose le cheval. Les bêtes tapent doucement. Il pose aussi un mouton. Elles sont bien, tes bêtes. La vache mange, papa. Et le mouton ? Il dort près de la vache. Aniss sort des perles. Elles sont rondes. Elles brillent un peu dans la lampe. Je fais un collier pour la vache. Un collier tout doux. Aniss enfile une perle. Puis une autre perle. Les perles font un tout petit bruit. Il pose le collier sur le cou de la vache. Elle est belle. Oui, elle est belle. Après, tu racontes une histoire, maman ? Oui, près de toi, au lit. La vache vient aussi. Maman s'approche du tapis. Le cheval bascule. Une perle roule. Le mouton glisse sur la vache. Oh. La ferme a bougé. Où est ma vache ? Sous le lit, peut-être ? Aniss se penche dans l'ombre. Le bois du lit est froid. Pas de vache. Dans le rond d'or ? Il cherche au milieu de la lumière. Des perles, le cheval, le mouton. Elle est perdue. J'ai besoin d'un petit coin, pour raconter. Je veux voir dessous. Aniss prend le cheval. Il le pose dans la caisse. Toc. La caisse sent le bois.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La fenêtre laisse entrer un air de terre mouillée, un peu froid. Un papillon de nuit se pose, puis frappe la vitre du bout des ailes. Sa silhouette tremble un peu, sur le tapis. Tu entends les ailes, Aniss ? Oui, maman. Le plancher craque sous le pas de papa. La lampe ronde est allumée. Elle chauffe le bois des bêtes, une à une. Sur le flanc de la vache, un &lt;emphasis level="moderate"&gt;éclat de lampe&lt;/emphasis&gt; brille. Il est tout petit, papa. C'est un éclat de lampe. La vache est lisse, un peu chaude sous le doigt. Le cheval sent le bois, sec et clair. C'est une ferme, maman. Une ferme sur le tapis. En ce moment, Aniss pose la vache au milieu du tapis. Il pose le cheval à côté, tap. Le mouton vient après, laine peinte, un peu rêche. Elles sont bien, tes bêtes. La vache mange, papa. Et le mouton ? Il dort près de la vache. Aniss sort des perles d'une coupelle. Elles sont rondes, un peu froides dans la paume. Je fais un collier, maintenant ! Pour la vache d'or ? Oui, et après l'histoire au lit. Aniss enfile une perle, clic. Puis une autre, clic, contre la première. Les perles font un tout petit bruit. Il pose le collier sur le cou de la vache. Elle est belle. Oui, elle est belle. L'histoire, maintenant, maman ! Près de toi, au lit ? La vache vient aussi. Maman s'approche du tapis, trop près des bêtes. Le cheval bascule. Une perle roule sous le lit. Le mouton glisse sur la vache, et la cache. Oh. La ferme a bougé. Où est ma vache ? Sous le lit, peut-être ? Aniss se penche dans l'ombre, près du bois. Le bois du lit est froid, un peu rugueux. Pas de vache. Dans le cercle de la lampe ? Il cherche au milieu de la lumière ronde. Des perles, le cheval, le mouton. Elle est perdue. Je prends tout, d'un coup ! Il saisit le cheval et le mouton trop vite. Les perles glissent entre ses doigts. Le tapis disparaît sous les bêtes. Ça ne veut pas, papa. Ses épaules tombent un peu. Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tu regardes sous les bêtes ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Éva joue dans sa chambre. Papa plie le linge près de la fenêtre. Éva a des animaux en bois. Elle fait une ferme. Les bêtes tapent doucement. Puis le jeu est fini. Papa dit : c'est l'heure de &lt;emphasis&gt;ranger&lt;/emphasis&gt;. Ranger, c'est remettre. Éva prend une vache. Elle la met dans la caisse. Elle prend un cheval. Elle le met dans la caisse. La caisse sent le bois. Plus tard, Éva sort des perles. Elle enfile un collier. Le jeu se termine encore. Éva se souvient. Elle range. Les perles vont dans la caisse. Le tapis redevient libre. Papa dit : après le jeu, on range. Les jouets retournent dans la caisse. Éva ferme le couvercle. Ça fait toc. Papa dit : merci Éva. [pause]</t>
+          <t>La fenêtre laisse entrer un air de terre mouillée, un peu froid. Un papillon de nuit se pose, puis frappe la vitre du bout des ailes. Sa silhouette tremble un peu, sur le tapis. Tu entends les ailes, Aniss ? Oui, maman. Le plancher craque sous le pas de papa. La lampe ronde est allumée. Elle chauffe le bois des bêtes, une à une. Sur le flanc de la vache, un &lt;emphasis&gt;éclat de lampe&lt;/emphasis&gt; brille. Il est tout petit, papa. C'est un éclat de lampe. La vache est lisse, un peu chaude sous le doigt. Le cheval sent le bois, sec et clair. C'est une ferme, maman. Une ferme sur le tapis. En ce moment, Aniss pose la vache au milieu du tapis. Il pose le cheval à côté, tap. Le mouton vient après, laine peinte, un peu rêche. Elles sont bien, tes bêtes. La vache mange, papa. Et le mouton ? Il dort près de la vache. Aniss sort des perles d'une coupelle. Elles sont rondes, un peu froides dans la paume. Je fais un collier, maintenant ! Pour la vache d'or ? Oui, et après l'histoire au lit. Aniss enfile une perle, clic. Puis une autre, clic, contre la première. Les perles font un tout petit bruit. Il pose le collier sur le cou de la vache. Elle est belle. Oui, elle est belle. L'histoire, maintenant, maman ! Près de toi, au lit ? La vache vient aussi. Maman s'approche du tapis, trop près des bêtes. Le cheval bascule. Une perle roule sous le lit. Le mouton glisse sur la vache, et la cache. Oh. La ferme a bougé. Où est ma vache ? Sous le lit, peut-être ? Aniss se penche dans l'ombre, près du bois. Le bois du lit est froid, un peu rugueux. Pas de vache. Dans le cercle de la lampe ? Il cherche au milieu de la lumière ronde. Des perles, le cheval, le mouton. Elle est perdue. Je prends tout, d'un coup ! Il saisit le cheval et le mouton trop vite. Les perles glissent entre ses doigts. Le tapis disparaît sous les bêtes. Ça ne veut pas, papa. Ses épaules tombent un peu. Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tu regardes sous les bêtes ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>ranger</t>
+          <t>éclat de lampe</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,66 +1321,79 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_la_vache_et_l_histoire_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un papillon de nuit frappe la vitre.
-narrateur|Tout doucement.
-narrateur|L'air sent la terre mouillée.
-narrateur|La fenêtre est un peu ouverte.
-narrateur|Le plancher craque.
-maman|Le soir est calme.
-papa|Oui, un petit soir doux.
-narrateur|Des animaux en bois attendent en rang.
-narrateur|La vache est lisse.
-narrateur|Le cheval sent le bois.
-narrateur|En ce moment, Aniss est à genoux.
-narrateur|Il est dans le rond d'or de la lampe.
+          <t>narrateur|La fenêtre laisse entrer un air de terre mouillée, un peu froid.
+narrateur|Un papillon de nuit se pose, puis frappe la vitre du bout des ailes.
+narrateur|Sa silhouette tremble un peu, sur le tapis.
+maman|Tu entends les ailes, Aniss ?
+enfant-m|Oui, maman.
+narrateur|Le plancher craque sous le pas de papa.
+papa|La lampe ronde est allumée.
+narrateur|Elle chauffe le bois des bêtes, une à une.
+narrateur|Sur le flanc de la vache, un éclat de lampe brille.
+enfant-m|Il est tout petit, papa.
+papa|C'est un éclat de lampe.
+narrateur|La vache est lisse, un peu chaude sous le doigt.
+narrateur|Le cheval sent le bois, sec et clair.
 enfant-m|C'est une ferme, maman.
 maman|Une ferme sur le tapis.
-narrateur|Aniss pose la vache.
-narrateur|Il pose le cheval.
-narrateur|Les bêtes tapent doucement.
-narrateur|Il pose aussi un mouton.
+narrateur|En ce moment, Aniss pose la vache au milieu du tapis.
+narrateur|Il pose le cheval à côté, tap.
+narrateur|Le mouton vient après, laine peinte, un peu rêche.
 papa|Elles sont bien, tes bêtes.
 enfant-m|La vache mange, papa.
 maman|Et le mouton ?
 enfant-m|Il dort près de la vache.
-narrateur|Aniss sort des perles.
-narrateur|Elles sont rondes.
-narrateur|Elles brillent un peu dans la lampe.
-enfant-m|Je fais un collier pour la vache.
-maman|Un collier tout doux.
-narrateur|Aniss enfile une perle.
-narrateur|Puis une autre perle.
+narrateur|Aniss sort des perles d'une coupelle.
+narrateur|Elles sont rondes, un peu froides dans la paume.
+enfant-m|Je fais un collier, maintenant !
+maman|Pour la vache d'or ?
+enfant-m|Oui, et après l'histoire au lit.
+narrateur|Aniss enfile une perle, clic.
+narrateur|Puis une autre, clic, contre la première.
 narrateur|Les perles font un tout petit bruit.
 narrateur|Il pose le collier sur le cou de la vache.
 enfant-m|Elle est belle.
 papa|Oui, elle est belle.
-enfant-m|Après, tu racontes une histoire, maman ?
-maman|Oui, près de toi, au lit.
+enfant-m|L'histoire, maintenant, maman !
+maman|Près de toi, au lit ?
 enfant-m|La vache vient aussi.
-narrateur|Maman s'approche du tapis.
+narrateur|Maman s'approche du tapis, trop près des bêtes.
 narrateur|Le cheval bascule.
-narrateur|Une perle roule.
-narrateur|Le mouton glisse sur la vache.
+narrateur|Une perle roule sous le lit.
+narrateur|Le mouton glisse sur la vache, et la cache.
 enfant-m|Oh.
 papa|La ferme a bougé.
 enfant-m|Où est ma vache ?
 maman|Sous le lit, peut-être ?
-narrateur|Aniss se penche dans l'ombre.
-narrateur|Le bois du lit est froid.
+narrateur|Aniss se penche dans l'ombre, près du bois.
+narrateur|Le bois du lit est froid, un peu rugueux.
 narrateur|Pas de vache.
-enfant-m|Dans le rond d'or ?
-narrateur|Il cherche au milieu de la lumière.
+enfant-m|Dans le cercle de la lampe ?
+narrateur|Il cherche au milieu de la lumière ronde.
 narrateur|Des perles, le cheval, le mouton.
 enfant-m|Elle est perdue.
-maman|J'ai besoin d'un petit coin, pour raconter.
-enfant-m|Je veux voir dessous.
-narrateur|Aniss prend le cheval.
-narrateur|Il le pose dans la caisse.
-narrateur|Toc.
-narrateur|La caisse sent le bois.</t>
+enfant-m|Je prends tout, d'un coup !
+narrateur|Il saisit le cheval et le mouton trop vite.
+narrateur|Les perles glissent entre ses doigts.
+narrateur|Le tapis disparaît sous les bêtes.
+enfant-m|Ça ne veut pas, papa.
+narrateur|Ses épaules tombent un peu.
+narrateur|Le sourire d'Aniss disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu regardes sous les bêtes ?</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>papillon,perles</t>
         </is>
       </c>
     </row>
@@ -1412,12 +1425,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Aniss cherche sa vache. Où est-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Aniss cherche sa &lt;emphasis level="moderate"&gt;vache&lt;/emphasis&gt;. Où est-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Après le jeu, que fait Éva ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Aniss cherche sa &lt;emphasis&gt;vache&lt;/emphasis&gt;. Où est-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1480,7 +1493,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1488,10 +1501,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1506,34 +1519,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>vache</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1542,23 +1559,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=la_vache_est_sous_le_mouton; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1591,17 +1608,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Le mouton va dans la caisse. Toc. Tu regardes bien sous les bêtes ? Oui, maman. Aniss ramasse une perle. Puis une autre. Elles cliquettent dans la caisse. Un bout de tapis reparaît. Sous le dernier mouton, un dos lisse. Ma vache ! La vache était sous le mouton. Le collier est encore autour du cou. Aniss la serre dans ses deux mains. Le bois est tiède, un peu lisse. Merci, tu l'as trouvée. Te voilà, petite vache. Elle dormait dessous. Les dernières perles vont dans la caisse. Le rond d'or est vide, au milieu. Le tapis est libre près du lit.</t>
+          <t>Aniss refuse de prendre toute la pile d'un coup. Il pose un genou au tapis, près des perles. Le cheval reste près de sa main. Je le mets tout seul. Il glisse le cheval dans la caisse. Toc. Le bois sent un peu la forêt. Tu regardes bien dessous ? Oui, maman. Un bout de tapis reparaît, gris et doux. Une perle va dans la caisse. Clic. Je sors le reste, d'un coup ! Il tire trop fort sur le mouton. Deux perles retombent, comme un petit toit. Oh. Il ne reprend pas trop vite. Il écoute la chambre, un instant. Sur le dos du mouton, l'éclat de lampe brille. Il est là. Aniss refuse de foncer. Il soulève le mouton, lentement. Un dos lisse, un peu chaud, apparaît. Ma vache ! La vache était sous le mouton. Le collier tient autour du cou. Aniss la serre contre sa joue. Merci, Aniss. Elle dormait dessous. La caisse a presque toutes les bêtes. Le tapis est libre, au milieu. On peut aller au lit ? Oui, avec la vache.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Le mouton va dans la caisse. Toc. Tu regardes bien sous les bêtes ? Oui, maman. Aniss ramasse une perle. Puis une autre. Elles cliquettent dans la caisse. Un bout de tapis reparaît. Sous le dernier mouton, un dos lisse. Ma vache ! La vache était sous le mouton. Le collier est encore autour du cou. Aniss la serre dans ses deux mains. Le bois est tiède, un peu lisse. Merci, tu l'as trouvée. Te voilà, petite vache. Elle dormait dessous. Les dernières perles vont dans la caisse. Le rond d'or est vide, au milieu. Le tapis est libre près du lit.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss refuse de prendre toute la pile d'un coup. Il pose un genou au tapis, près des perles. Le cheval reste près de sa main. Je le mets tout seul. Il glisse le cheval dans la caisse. Toc. Le bois sent un peu la forêt. Tu regardes bien dessous ? Oui, maman. Un bout de tapis reparaît, gris et doux. Une perle va dans la caisse. Clic. Je sors le reste, d'un coup ! Il tire trop fort sur le mouton. Deux perles retombent, comme un petit toit. Oh. Il ne reprend pas trop vite. Il écoute la chambre, un instant. Sur le dos du mouton, l'&lt;emphasis level="moderate"&gt;éclat de lampe&lt;/emphasis&gt; brille. Il est là. Aniss refuse de foncer. Il soulève le mouton, lentement. Un dos lisse, un peu chaud, apparaît. Ma vache ! La vache était sous le mouton. Le collier tient autour du cou. Aniss la serre contre sa joue. Merci, Aniss. Elle dormait dessous. La caisse a presque toutes les bêtes. Le tapis est libre, au milieu. On peut aller au lit ? Oui, avec la vache.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Éva a rangé. Les jouets sont dans la &lt;emphasis&gt;caisse&lt;/emphasis&gt;. Le tapis est libre. Papa est là. [pause]</t>
+          <t>Aniss refuse de prendre toute la pile d'un coup. Il pose un genou au tapis, près des perles. Le cheval reste près de sa main. Je le mets tout seul. Il glisse le cheval dans la caisse. Toc. Le bois sent un peu la forêt. Tu regardes bien dessous ? Oui, maman. Un bout de tapis reparaît, gris et doux. Une perle va dans la caisse. Clic. Je sors le reste, d'un coup ! Il tire trop fort sur le mouton. Deux perles retombent, comme un petit toit. Oh. Il ne reprend pas trop vite. Il écoute la chambre, un instant. Sur le dos du mouton, l'&lt;emphasis&gt;éclat de lampe&lt;/emphasis&gt; brille. Il est là. Aniss refuse de foncer. Il soulève le mouton, lentement. Un dos lisse, un peu chaud, apparaît. Ma vache ! La vache était sous le mouton. Le collier tient autour du cou. Aniss la serre contre sa joue. Merci, Aniss. Elle dormait dessous. La caisse a presque toutes les bêtes. Le tapis est libre, au milieu. On peut aller au lit ? Oui, avec la vache. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1648,7 +1665,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1656,10 +1673,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1682,30 +1699,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>caisse</t>
+          <t>éclat de lampe</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1714,10 +1731,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1730,31 +1747,49 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=concentration puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_pose_une_bete_sans_foncer; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Le mouton va dans la caisse.
+          <t>narrateur|Aniss refuse de prendre toute la pile d'un coup.
+narrateur|Il pose un genou au tapis, près des perles.
+narrateur|Le cheval reste près de sa main.
+enfant-m|Je le mets tout seul.
+narrateur|Il glisse le cheval dans la caisse.
 narrateur|Toc.
-maman|Tu regardes bien sous les bêtes ?
+narrateur|Le bois sent un peu la forêt.
+maman|Tu regardes bien dessous ?
 enfant-m|Oui, maman.
-narrateur|Aniss ramasse une perle.
-narrateur|Puis une autre.
-narrateur|Elles cliquettent dans la caisse.
-papa|Un bout de tapis reparaît.
-narrateur|Sous le dernier mouton, un dos lisse.
+narrateur|Un bout de tapis reparaît, gris et doux.
+narrateur|Une perle va dans la caisse.
+narrateur|Clic.
+enfant-m|Je sors le reste, d'un coup !
+narrateur|Il tire trop fort sur le mouton.
+narrateur|Deux perles retombent, comme un petit toit.
+enfant-m|Oh.
+narrateur|Il ne reprend pas trop vite.
+narrateur|Il écoute la chambre, un instant.
+narrateur|Sur le dos du mouton, l'éclat de lampe brille.
+enfant-m|Il est là.
+narrateur|Aniss refuse de foncer.
+narrateur|Il soulève le mouton, lentement.
+narrateur|Un dos lisse, un peu chaud, apparaît.
 enfant-m|Ma vache !
 narrateur|La vache était sous le mouton.
-narrateur|Le collier est encore autour du cou.
-narrateur|Aniss la serre dans ses deux mains.
-narrateur|Le bois est tiède, un peu lisse.
-papa|Merci, tu l'as trouvée.
-maman|Te voilà, petite vache.
+narrateur|Le collier tient autour du cou.
+narrateur|Aniss la serre contre sa joue.
+papa|Merci, Aniss.
 enfant-m|Elle dormait dessous.
-narrateur|Les dernières perles vont dans la caisse.
-narrateur|Le rond d'or est vide, au milieu.
-narrateur|Le tapis est libre près du lit.</t>
+narrateur|La caisse a presque toutes les bêtes.
+narrateur|Le tapis est libre, au milieu.
+maman|On peut aller au lit ?
+enfant-m|Oui, avec la vache.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>caisse,bois</t>
         </is>
       </c>
     </row>
@@ -1781,17 +1816,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Aniss grimpe sur le lit. La vache est sur la couverture. Le collier brille un peu. Je m'assoie ? Oui, maman. Maman s'assoit au bord. Sa voix est basse, tout près. Tu veux un verre d'eau, avant ? Une gorgée, papa. L'eau est tiède. Aniss pose la vache contre l'oreiller. Le papillon de nuit repose sur la vitre. On écoute l'histoire, maintenant. La vache écoute aussi. Oui, tout le monde écoute. La lampe fait encore son rond d'or. L'air sent la terre mouillée.</t>
+          <t>Tu grimpes avec elle ? Aniss grimpe sur le lit, la vache dans la main. La vache est sur la couverture. Le collier brille un peu, près du genou. Je m'assoie ? Oui, maman. Maman s'assoit au bord, près de l'oreiller. Sa voix est basse, près de lui. Tu veux un peu d'eau ? Une gorgée, papa. L'eau est tiède. Aniss pose la vache contre l'oreiller. Je tire la couverture ! Aniss s'arrête. Il refuse de foncer. Il recule le pli, lentement. La couverture se pose, plate. L'histoire peut s'asseoir. Le papillon de nuit repose sur la vitre. On écoute, maintenant. La vache écoute aussi. Oui, on écoute avec elle. La lampe tient son cercle chaud. L'air sent la terre mouillée.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Aniss grimpe sur le lit. La vache est sur la couverture. Le collier brille un peu. Je m'assoie ? Oui, maman. Maman s'assoit au bord. Sa voix est basse, tout près. Tu veux un verre d'eau, avant ? Une gorgée, papa. L'eau est tiède. Aniss pose la vache contre l'oreiller. Le papillon de nuit repose sur la vitre. On écoute l'histoire, maintenant. La vache écoute aussi. Oui, tout le monde écoute. La lampe fait encore son rond d'or. L'air sent la terre mouillée.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tu grimpes avec elle ? Aniss grimpe sur le lit, la vache dans la main. La vache est sur la &lt;emphasis level="moderate"&gt;couverture&lt;/emphasis&gt;. Le collier brille un peu, près du genou. Je m'assoie ? Oui, maman. Maman s'assoit au bord, près de l'oreiller. Sa voix est basse, près de lui. Tu veux un peu d'eau ? Une gorgée, papa. L'eau est tiède. Aniss pose la vache contre l'oreiller. Je tire la couverture ! Aniss s'arrête. Il refuse de foncer. Il recule le pli, lentement. La couverture se pose, plate. L'histoire peut s'asseoir. Le papillon de nuit repose sur la vitre. On écoute, maintenant. La vache écoute aussi. Oui, on écoute avec elle. La lampe tient son cercle chaud. L'air sent la terre mouillée.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Éva pousse la &lt;emphasis&gt;caisse&lt;/emphasis&gt; sous le lit. Papa tend un verre d'eau. [pause]</t>
+          <t>Tu grimpes avec elle ? Aniss grimpe sur le lit, la vache dans la main. La vache est sur la &lt;emphasis&gt;couverture&lt;/emphasis&gt;. Le collier brille un peu, près du genou. Je m'assoie ? Oui, maman. Maman s'assoit au bord, près de l'oreiller. Sa voix est basse, près de lui. Tu veux un peu d'eau ? Une gorgée, papa. L'eau est tiède. Aniss pose la vache contre l'oreiller. Je tire la couverture ! Aniss s'arrête. Il refuse de foncer. Il recule le pli, lentement. La couverture se pose, plate. L'histoire peut s'asseoir. Le papillon de nuit repose sur la vitre. On écoute, maintenant. La vache écoute aussi. Oui, on écoute avec elle. La lampe tient son cercle chaud. L'air sent la terre mouillée. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1838,7 +1873,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1846,10 +1881,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1872,30 +1907,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>caisse</t>
+          <t>couverture</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1904,10 +1939,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1918,26 +1953,42 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_tirer_la_couverture; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Aniss grimpe sur le lit.
+          <t>papa|Tu grimpes avec elle ?
+narrateur|Aniss grimpe sur le lit, la vache dans la main.
 narrateur|La vache est sur la couverture.
-narrateur|Le collier brille un peu.
+narrateur|Le collier brille un peu, près du genou.
 maman|Je m'assoie ?
 enfant-m|Oui, maman.
-narrateur|Maman s'assoit au bord.
-narrateur|Sa voix est basse, tout près.
-papa|Tu veux un verre d'eau, avant ?
+narrateur|Maman s'assoit au bord, près de l'oreiller.
+narrateur|Sa voix est basse, près de lui.
+papa|Tu veux un peu d'eau ?
 enfant-m|Une gorgée, papa.
 narrateur|L'eau est tiède.
 narrateur|Aniss pose la vache contre l'oreiller.
+enfant-m|Je tire la couverture !
+narrateur|Aniss s'arrête.
+narrateur|Il refuse de foncer.
+narrateur|Il recule le pli, lentement.
+narrateur|La couverture se pose, plate.
+papa|L'histoire peut s'asseoir.
 narrateur|Le papillon de nuit repose sur la vitre.
-maman|On écoute l'histoire, maintenant.
+maman|On écoute, maintenant.
 enfant-m|La vache écoute aussi.
-papa|Oui, tout le monde écoute.
-narrateur|La lampe fait encore son rond d'or.
+papa|Oui, on écoute avec elle.
+narrateur|La lampe tient son cercle chaud.
 narrateur|L'air sent la terre mouillée.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>couverture,eau</t>
         </is>
       </c>
     </row>
@@ -1964,17 +2015,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>La vache est sur l'oreiller. Toi aussi, tu es bien. Bravo, tu l'as retrouvée. Le papillon repose ses ailes. Le rond d'or reste sur la couverture.</t>
+          <t>Ils s'assoient près de la couverture tiède. La chaleur touche les joues d'Aniss. La vache est là. Oui, près de toi. Le collier tient un tout petit reflet. Comme l'éclat de lampe, papa ! Tu le vois, toi ? Oui, sur le flanc. Aniss glisse la vache sans se presser. Le bois repose contre sa hanche. On le sent, maman. Tu le sens sur tes joues ? Oui, il est chaud. Le papillon repose ses ailes. L'éclat de lampe tient sur le flanc.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>La vache est sur l'oreiller. Toi aussi, tu es bien. Bravo, tu l'as retrouvée. Le papillon repose ses ailes. Le rond d'or reste sur la couverture.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils s'assoient près de la couverture tiède. La chaleur touche les joues d'Aniss. La vache est là. Oui, près de toi. Le collier tient un tout petit reflet. Comme l'&lt;emphasis level="moderate"&gt;éclat de lampe&lt;/emphasis&gt;, papa ! Tu le vois, toi ? Oui, sur le flanc. Aniss glisse la vache sans se presser. Le bois repose contre sa hanche. On le sent, maman. Tu le sens sur tes joues ? Oui, il est chaud. Le papillon repose ses ailes. L'éclat de lampe tient sur le flanc.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils s'assoient près de la couverture tiède. La chaleur touche les joues d'Aniss. La vache est là. Oui, près de toi. Le collier tient un tout petit reflet. Comme l'&lt;emphasis&gt;éclat de lampe&lt;/emphasis&gt;, papa ! Tu le vois, toi ? Oui, sur le flanc. Aniss glisse la vache sans se presser. Le bois repose contre sa hanche. On le sent, maman. Tu le sens sur tes joues ? Oui, il est chaud. Le papillon repose ses ailes. L'éclat de lampe tient sur le flanc.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2021,18 +2072,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2041,12 +2092,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2055,17 +2106,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de lampe</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2074,11 +2129,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2087,28 +2142,47 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_flanc; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|La vache est sur l'oreiller.
-maman|Toi aussi, tu es bien.
-papa|Bravo, tu l'as retrouvée.
+          <t>narrateur|Ils s'assoient près de la couverture tiède.
+narrateur|La chaleur touche les joues d'Aniss.
+enfant-m|La vache est là.
+maman|Oui, près de toi.
+narrateur|Le collier tient un tout petit reflet.
+enfant-m|Comme l'éclat de lampe, papa !
+papa|Tu le vois, toi ?
+enfant-m|Oui, sur le flanc.
+narrateur|Aniss glisse la vache sans se presser.
+narrateur|Le bois repose contre sa hanche.
+enfant-m|On le sent, maman.
+maman|Tu le sens sur tes joues ?
+enfant-m|Oui, il est chaud.
 narrateur|Le papillon repose ses ailes.
-narrateur|Le rond d'or reste sur la couverture.</t>
+narrateur|L'éclat de lampe tient sur le flanc.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>lampe,vache</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2203,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2221,6 +2295,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>